<commit_message>
Updated files to create person-specific roster and shift schedule templates
</commit_message>
<xml_diff>
--- a/outputs/rotation_v0.xlsx
+++ b/outputs/rotation_v0.xlsx
@@ -3402,54 +3402,54 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>OPERATIONAL</t>
+          <t>POST-CLOSE</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr"/>
-      <c r="E29" s="8" t="inlineStr">
-        <is>
-          <t>First Aid</t>
-        </is>
-      </c>
-      <c r="F29" s="8" t="inlineStr">
-        <is>
-          <t>Left Shore</t>
-        </is>
-      </c>
-      <c r="G29" s="8" t="inlineStr">
-        <is>
-          <t>Right Shore</t>
-        </is>
-      </c>
-      <c r="H29" s="8" t="inlineStr">
-        <is>
-          <t>Floater</t>
-        </is>
-      </c>
-      <c r="I29" s="8" t="inlineStr">
-        <is>
-          <t>Rental</t>
-        </is>
-      </c>
-      <c r="J29" s="8" t="inlineStr">
-        <is>
-          <t>Tower</t>
-        </is>
-      </c>
-      <c r="K29" s="8" t="inlineStr">
-        <is>
-          <t>Left Reef</t>
-        </is>
-      </c>
-      <c r="L29" s="8" t="inlineStr">
-        <is>
-          <t>Right Reef</t>
-        </is>
-      </c>
-      <c r="M29" s="8" t="inlineStr">
-        <is>
-          <t>Floater</t>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="I29" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="J29" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="K29" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="L29" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="M29" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
         </is>
       </c>
       <c r="N29" s="7" t="inlineStr">
@@ -6443,54 +6443,54 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>OPERATIONAL</t>
+          <t>POST-CLOSE</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr"/>
-      <c r="E29" s="8" t="inlineStr">
-        <is>
-          <t>First Aid</t>
-        </is>
-      </c>
-      <c r="F29" s="8" t="inlineStr">
-        <is>
-          <t>Left Shore</t>
-        </is>
-      </c>
-      <c r="G29" s="8" t="inlineStr">
-        <is>
-          <t>Right Shore</t>
-        </is>
-      </c>
-      <c r="H29" s="8" t="inlineStr">
-        <is>
-          <t>Floater</t>
-        </is>
-      </c>
-      <c r="I29" s="8" t="inlineStr">
-        <is>
-          <t>Rental</t>
-        </is>
-      </c>
-      <c r="J29" s="8" t="inlineStr">
-        <is>
-          <t>Tower</t>
-        </is>
-      </c>
-      <c r="K29" s="8" t="inlineStr">
-        <is>
-          <t>Left Reef</t>
-        </is>
-      </c>
-      <c r="L29" s="8" t="inlineStr">
-        <is>
-          <t>Right Reef</t>
-        </is>
-      </c>
-      <c r="M29" s="8" t="inlineStr">
-        <is>
-          <t>Floater</t>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="I29" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="J29" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="K29" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="L29" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="M29" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
         </is>
       </c>
       <c r="N29" s="7" t="inlineStr">
@@ -9484,54 +9484,54 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>OPERATIONAL</t>
+          <t>POST-CLOSE</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr"/>
-      <c r="E29" s="8" t="inlineStr">
-        <is>
-          <t>First Aid</t>
-        </is>
-      </c>
-      <c r="F29" s="8" t="inlineStr">
-        <is>
-          <t>Left Shore</t>
-        </is>
-      </c>
-      <c r="G29" s="8" t="inlineStr">
-        <is>
-          <t>Right Shore</t>
-        </is>
-      </c>
-      <c r="H29" s="8" t="inlineStr">
-        <is>
-          <t>Floater</t>
-        </is>
-      </c>
-      <c r="I29" s="8" t="inlineStr">
-        <is>
-          <t>Rental</t>
-        </is>
-      </c>
-      <c r="J29" s="8" t="inlineStr">
-        <is>
-          <t>Tower</t>
-        </is>
-      </c>
-      <c r="K29" s="8" t="inlineStr">
-        <is>
-          <t>Left Reef</t>
-        </is>
-      </c>
-      <c r="L29" s="8" t="inlineStr">
-        <is>
-          <t>Right Reef</t>
-        </is>
-      </c>
-      <c r="M29" s="8" t="inlineStr">
-        <is>
-          <t>Floater</t>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="I29" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="J29" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="K29" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="L29" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="M29" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
         </is>
       </c>
       <c r="N29" s="7" t="inlineStr">
@@ -12525,54 +12525,54 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>OPERATIONAL</t>
+          <t>POST-CLOSE</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr"/>
-      <c r="E29" s="8" t="inlineStr">
-        <is>
-          <t>First Aid</t>
-        </is>
-      </c>
-      <c r="F29" s="8" t="inlineStr">
-        <is>
-          <t>Left Shore</t>
-        </is>
-      </c>
-      <c r="G29" s="8" t="inlineStr">
-        <is>
-          <t>Right Shore</t>
-        </is>
-      </c>
-      <c r="H29" s="8" t="inlineStr">
-        <is>
-          <t>Floater</t>
-        </is>
-      </c>
-      <c r="I29" s="8" t="inlineStr">
-        <is>
-          <t>Rental</t>
-        </is>
-      </c>
-      <c r="J29" s="8" t="inlineStr">
-        <is>
-          <t>Tower</t>
-        </is>
-      </c>
-      <c r="K29" s="8" t="inlineStr">
-        <is>
-          <t>Left Reef</t>
-        </is>
-      </c>
-      <c r="L29" s="8" t="inlineStr">
-        <is>
-          <t>Right Reef</t>
-        </is>
-      </c>
-      <c r="M29" s="8" t="inlineStr">
-        <is>
-          <t>Floater</t>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="I29" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="J29" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="K29" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="L29" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="M29" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
         </is>
       </c>
       <c r="N29" s="7" t="inlineStr">
@@ -15780,54 +15780,54 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>OPERATIONAL</t>
+          <t>POST-CLOSE</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr"/>
-      <c r="E31" s="8" t="inlineStr">
-        <is>
-          <t>Left Shore</t>
-        </is>
-      </c>
-      <c r="F31" s="8" t="inlineStr">
-        <is>
-          <t>Right Shore</t>
-        </is>
-      </c>
-      <c r="G31" s="8" t="inlineStr">
-        <is>
-          <t>First Aid</t>
-        </is>
-      </c>
-      <c r="H31" s="8" t="inlineStr">
-        <is>
-          <t>Floater</t>
-        </is>
-      </c>
-      <c r="I31" s="8" t="inlineStr">
-        <is>
-          <t>Tower</t>
-        </is>
-      </c>
-      <c r="J31" s="8" t="inlineStr">
-        <is>
-          <t>Left Reef</t>
-        </is>
-      </c>
-      <c r="K31" s="8" t="inlineStr">
-        <is>
-          <t>Right Reef</t>
-        </is>
-      </c>
-      <c r="L31" s="8" t="inlineStr">
-        <is>
-          <t>Rental</t>
-        </is>
-      </c>
-      <c r="M31" s="8" t="inlineStr">
-        <is>
-          <t>Floater</t>
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="G31" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="I31" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="J31" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="K31" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="L31" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="M31" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
         </is>
       </c>
       <c r="N31" s="7" t="inlineStr">
@@ -19249,54 +19249,54 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>OPERATIONAL</t>
+          <t>POST-CLOSE</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr"/>
-      <c r="E33" s="8" t="inlineStr">
-        <is>
-          <t>Right Shore</t>
-        </is>
-      </c>
-      <c r="F33" s="8" t="inlineStr">
-        <is>
-          <t>First Aid</t>
-        </is>
-      </c>
-      <c r="G33" s="8" t="inlineStr">
-        <is>
-          <t>Left Shore</t>
-        </is>
-      </c>
-      <c r="H33" s="8" t="inlineStr">
-        <is>
-          <t>Floater</t>
-        </is>
-      </c>
-      <c r="I33" s="8" t="inlineStr">
-        <is>
-          <t>Left Reef</t>
-        </is>
-      </c>
-      <c r="J33" s="8" t="inlineStr">
-        <is>
-          <t>Right Reef</t>
-        </is>
-      </c>
-      <c r="K33" s="8" t="inlineStr">
-        <is>
-          <t>Rental</t>
-        </is>
-      </c>
-      <c r="L33" s="8" t="inlineStr">
-        <is>
-          <t>Tower</t>
-        </is>
-      </c>
-      <c r="M33" s="8" t="inlineStr">
-        <is>
-          <t>Floater</t>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="F33" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="H33" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="I33" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="J33" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="K33" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="L33" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="M33" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
         </is>
       </c>
       <c r="N33" s="7" t="inlineStr">
@@ -22504,54 +22504,54 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>OPERATIONAL</t>
+          <t>POST-CLOSE</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr"/>
-      <c r="E31" s="8" t="inlineStr">
-        <is>
-          <t>Left Shore</t>
-        </is>
-      </c>
-      <c r="F31" s="8" t="inlineStr">
-        <is>
-          <t>Right Shore</t>
-        </is>
-      </c>
-      <c r="G31" s="8" t="inlineStr">
-        <is>
-          <t>First Aid</t>
-        </is>
-      </c>
-      <c r="H31" s="8" t="inlineStr">
-        <is>
-          <t>Floater</t>
-        </is>
-      </c>
-      <c r="I31" s="8" t="inlineStr">
-        <is>
-          <t>Tower</t>
-        </is>
-      </c>
-      <c r="J31" s="8" t="inlineStr">
-        <is>
-          <t>Left Reef</t>
-        </is>
-      </c>
-      <c r="K31" s="8" t="inlineStr">
-        <is>
-          <t>Right Reef</t>
-        </is>
-      </c>
-      <c r="L31" s="8" t="inlineStr">
-        <is>
-          <t>Rental</t>
-        </is>
-      </c>
-      <c r="M31" s="8" t="inlineStr">
-        <is>
-          <t>Floater</t>
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="G31" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="I31" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="J31" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="K31" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="L31" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="M31" s="7" t="inlineStr">
+        <is>
+          <t>OFF</t>
         </is>
       </c>
       <c r="N31" s="7" t="inlineStr">

</xml_diff>